<commit_message>
test driven python lib Krippendorff
</commit_message>
<xml_diff>
--- a/materials/25_random_scenario_judgement_adya.xlsx
+++ b/materials/25_random_scenario_judgement_adya.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="282">
   <si>
     <t>paper_id</t>
   </si>
@@ -92,7 +92,7 @@
     <t>because it mentioned 'AI system' which is essentially a actor</t>
   </si>
   <si>
-    <t>Not Specified</t>
+    <t>Not specified</t>
   </si>
   <si>
     <t>any intended or resultant harmful activity not found. The capability of broad congnitive tasks may be in focus but it not conveying any sense of threat or future threat</t>
@@ -518,9 +518,6 @@
   </si>
   <si>
     <t>fact of independent goal seeking AGI</t>
-  </si>
-  <si>
-    <t>Not specified</t>
   </si>
   <si>
     <t>it talk about AI target not Knowledge</t>
@@ -2162,28 +2159,28 @@
         <v>165</v>
       </c>
       <c r="K15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="L15" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>24</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O15" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P15" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R15" s="11" t="s">
         <v>169</v>
-      </c>
-      <c r="Q15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R15" s="11" t="s">
-        <v>170</v>
       </c>
       <c r="S15" s="12"/>
       <c r="T15" s="12"/>
@@ -2194,58 +2191,58 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>174</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>24</v>
       </c>
       <c r="H16" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J16" s="8" t="s">
+      <c r="K16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L16" s="8" t="s">
         <v>176</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L16" s="8" t="s">
-        <v>177</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P16" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="R16" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="S16" s="12"/>
       <c r="T16" s="12"/>
@@ -2256,16 +2253,16 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>183</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>22</v>
@@ -2277,37 +2274,37 @@
         <v>22</v>
       </c>
       <c r="H17" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>184</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>185</v>
       </c>
       <c r="K17" s="9" t="s">
         <v>63</v>
       </c>
       <c r="L17" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="M17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N17" s="8" t="s">
+      <c r="O17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P17" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="O17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="P17" s="8" t="s">
+      <c r="Q17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R17" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="Q17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R17" s="11" t="s">
-        <v>189</v>
       </c>
       <c r="S17" s="12"/>
       <c r="T17" s="12"/>
@@ -2318,58 +2315,58 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F18" s="8" t="s">
+      <c r="G18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H18" s="8" t="s">
+      <c r="I18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J18" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J18" s="8" t="s">
+      <c r="K18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L18" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="K18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L18" s="8" t="s">
+      <c r="M18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N18" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="M18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N18" s="8" t="s">
+      <c r="O18" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="P18" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="O18" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="P18" s="10" t="s">
+      <c r="Q18" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="R18" s="13" t="s">
         <v>198</v>
-      </c>
-      <c r="Q18" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="R18" s="13" t="s">
-        <v>199</v>
       </c>
       <c r="S18" s="12"/>
       <c r="T18" s="12"/>
@@ -2380,58 +2377,58 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>202</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>203</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>36</v>
       </c>
       <c r="H19" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J19" s="8" t="s">
         <v>204</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>205</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>63</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="O19" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P19" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q19" s="7" t="s">
         <v>24</v>
       </c>
       <c r="R19" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="S19" s="12"/>
       <c r="T19" s="12"/>
@@ -2442,58 +2439,58 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" s="8" t="s">
+      <c r="G20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="G20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="8" t="s">
+      <c r="I20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J20" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J20" s="8" t="s">
+      <c r="K20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="8" t="s">
         <v>215</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="L20" s="8" t="s">
-        <v>216</v>
       </c>
       <c r="M20" s="9" t="s">
         <v>24</v>
       </c>
       <c r="N20" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P20" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="O20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="P20" s="8" t="s">
+      <c r="Q20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R20" s="11" t="s">
         <v>218</v>
-      </c>
-      <c r="Q20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R20" s="11" t="s">
-        <v>219</v>
       </c>
       <c r="S20" s="12"/>
       <c r="T20" s="12"/>
@@ -2504,16 +2501,16 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>221</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>222</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>22</v>
@@ -2525,37 +2522,37 @@
         <v>22</v>
       </c>
       <c r="H21" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21" s="8" t="s">
+      <c r="K21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L21" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="K21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L21" s="8" t="s">
+      <c r="M21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N21" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="M21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N21" s="8" t="s">
+      <c r="O21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P21" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="O21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="P21" s="8" t="s">
+      <c r="Q21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R21" s="11" t="s">
         <v>227</v>
-      </c>
-      <c r="Q21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R21" s="11" t="s">
-        <v>228</v>
       </c>
       <c r="S21" s="12"/>
       <c r="T21" s="12"/>
@@ -2566,58 +2563,58 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" s="8" t="s">
+      <c r="G22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="G22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="8" t="s">
+      <c r="I22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J22" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J22" s="8" t="s">
+      <c r="K22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L22" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="K22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L22" s="8" t="s">
+      <c r="M22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N22" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="M22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N22" s="8" t="s">
+      <c r="O22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P22" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="O22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="P22" s="8" t="s">
+      <c r="Q22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R22" s="11" t="s">
         <v>237</v>
-      </c>
-      <c r="Q22" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R22" s="11" t="s">
-        <v>238</v>
       </c>
       <c r="S22" s="12"/>
       <c r="T22" s="12"/>
@@ -2628,58 +2625,58 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>240</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>241</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>24</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>24</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>24</v>
       </c>
       <c r="J23" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="8" t="s">
         <v>244</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="L23" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="M23" s="7" t="s">
         <v>24</v>
       </c>
       <c r="N23" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="O23" s="7" t="s">
         <v>63</v>
       </c>
       <c r="P23" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Q23" s="7" t="s">
         <v>24</v>
       </c>
       <c r="R23" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="S23" s="12"/>
       <c r="T23" s="12"/>
@@ -2690,58 +2687,58 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24" s="8" t="s">
+      <c r="G24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="G24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="8" t="s">
+      <c r="I24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J24" s="8" t="s">
+      <c r="K24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L24" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="K24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L24" s="8" t="s">
+      <c r="M24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N24" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="M24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N24" s="8" t="s">
-        <v>256</v>
       </c>
       <c r="O24" s="9" t="s">
         <v>63</v>
       </c>
       <c r="P24" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R24" s="11" t="s">
         <v>257</v>
-      </c>
-      <c r="Q24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R24" s="11" t="s">
-        <v>258</v>
       </c>
       <c r="S24" s="12"/>
       <c r="T24" s="12"/>
@@ -2752,16 +2749,16 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>260</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>261</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>22</v>
@@ -2773,37 +2770,37 @@
         <v>22</v>
       </c>
       <c r="H25" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="8" t="s">
+      <c r="K25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L25" s="8" t="s">
         <v>263</v>
-      </c>
-      <c r="K25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>264</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>63</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O25" s="7" t="s">
         <v>63</v>
       </c>
       <c r="P25" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R25" s="11" t="s">
         <v>266</v>
-      </c>
-      <c r="Q25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R25" s="11" t="s">
-        <v>267</v>
       </c>
       <c r="S25" s="12"/>
       <c r="T25" s="12"/>
@@ -2814,58 +2811,58 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F26" s="8" t="s">
+      <c r="G26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="G26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="8" t="s">
+      <c r="I26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="8" t="s">
+      <c r="K26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L26" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="K26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L26" s="8" t="s">
+      <c r="M26" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="N26" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="M26" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="N26" s="10" t="s">
+      <c r="O26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P26" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="O26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="P26" s="8" t="s">
+      <c r="Q26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="R26" s="11" t="s">
         <v>276</v>
-      </c>
-      <c r="Q26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="R26" s="11" t="s">
-        <v>277</v>
       </c>
       <c r="S26" s="12"/>
       <c r="T26" s="12"/>
@@ -4039,7 +4036,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B1" s="24">
         <v>16.0</v>
@@ -4047,7 +4044,7 @@
     </row>
     <row r="2">
       <c r="A2" s="24" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B2" s="24">
         <v>29.0</v>
@@ -4055,15 +4052,15 @@
     </row>
     <row r="3">
       <c r="A3" s="24" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" s="25" t="s">
         <v>280</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="24" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B4" s="24">
         <v>175.0</v>

</xml_diff>